<commit_message>
xử lý ca liền
</commit_message>
<xml_diff>
--- a/convert/baocao1.xlsx
+++ b/convert/baocao1.xlsx
@@ -81938,7 +81938,7 @@
         <v>4</v>
       </c>
       <c r="BK415" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="BL415">
         <v>1.5</v>
@@ -110209,7 +110209,7 @@
         <v>4</v>
       </c>
       <c r="BK566" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="BL566">
         <v>1.5</v>

</xml_diff>